<commit_message>
Actualizacion datos REM 2026-07-22 16:41 (orquestador)
</commit_message>
<xml_diff>
--- a/output/2025_A03_SECCION_A5_TABLAS.xlsx
+++ b/output/2025_A03_SECCION_A5_TABLAS.xlsx
@@ -195,6 +195,9 @@
     <t>nombre_establecimiento</t>
   </si>
   <si>
+    <t>CECOSF Wilma Yoli Gomez Conejera</t>
+  </si>
+  <si>
     <t>Centro Comunitario de Salud Familiar Alberto Bachelet</t>
   </si>
   <si>
@@ -274,9 +277,6 @@
   </si>
   <si>
     <t>Centro Comunitario de Salud Familiar Las Lomas</t>
-  </si>
-  <si>
-    <t>Centro Comunitario de Salud Familiar Lo Chacón</t>
   </si>
   <si>
     <t>Centro Comunitario de Salud Familiar Lo Errázuriz</t>
@@ -2041,13 +2041,13 @@
         <v>57</v>
       </c>
       <c r="B3">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C3">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D3">
-        <v>43.90243902439025</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2055,10 +2055,13 @@
         <v>58</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>41</v>
+      </c>
+      <c r="D4">
+        <v>43.90243902439025</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2066,13 +2069,10 @@
         <v>59</v>
       </c>
       <c r="B5">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="C5">
-        <v>12</v>
-      </c>
-      <c r="D5">
-        <v>91.66666666666666</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2080,13 +2080,13 @@
         <v>60</v>
       </c>
       <c r="B6">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="C6">
-        <v>69</v>
+        <v>12</v>
       </c>
       <c r="D6">
-        <v>65.21739130434783</v>
+        <v>91.66666666666666</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2094,13 +2094,13 @@
         <v>61</v>
       </c>
       <c r="B7">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C7">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="D7">
-        <v>90.90909090909091</v>
+        <v>65.21739130434783</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2108,13 +2108,13 @@
         <v>62</v>
       </c>
       <c r="B8">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C8">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D8">
-        <v>70.58823529411765</v>
+        <v>90.90909090909091</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2122,13 +2122,13 @@
         <v>63</v>
       </c>
       <c r="B9">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C9">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D9">
-        <v>58.33333333333334</v>
+        <v>70.58823529411765</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2136,13 +2136,13 @@
         <v>64</v>
       </c>
       <c r="B10">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C10">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="D10">
-        <v>80.95238095238095</v>
+        <v>58.33333333333334</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2150,13 +2150,13 @@
         <v>65</v>
       </c>
       <c r="B11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D11">
-        <v>94.11764705882352</v>
+        <v>80.95238095238095</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2164,13 +2164,13 @@
         <v>66</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>94.11764705882352</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2178,13 +2178,13 @@
         <v>67</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C13">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D13">
-        <v>57.14285714285714</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2192,13 +2192,13 @@
         <v>68</v>
       </c>
       <c r="B14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D14">
-        <v>75</v>
+        <v>57.14285714285714</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2206,13 +2206,13 @@
         <v>69</v>
       </c>
       <c r="B15">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="C15">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="D15">
-        <v>67.3469387755102</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2220,13 +2220,13 @@
         <v>70</v>
       </c>
       <c r="B16">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="C16">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="D16">
-        <v>62.5</v>
+        <v>67.3469387755102</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2234,13 +2234,13 @@
         <v>71</v>
       </c>
       <c r="B17">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C17">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D17">
-        <v>73.68421052631578</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2248,13 +2248,13 @@
         <v>72</v>
       </c>
       <c r="B18">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C18">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D18">
-        <v>76.92307692307693</v>
+        <v>73.68421052631578</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2262,13 +2262,13 @@
         <v>73</v>
       </c>
       <c r="B19">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C19">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D19">
-        <v>66.66666666666666</v>
+        <v>76.92307692307693</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2276,10 +2276,13 @@
         <v>74</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="D20">
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2287,13 +2290,10 @@
         <v>75</v>
       </c>
       <c r="B21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21">
-        <v>5</v>
-      </c>
-      <c r="D21">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2301,13 +2301,13 @@
         <v>76</v>
       </c>
       <c r="B22">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C22">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D22">
-        <v>80</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2315,10 +2315,13 @@
         <v>77</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="D23">
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2329,9 +2332,6 @@
         <v>0</v>
       </c>
       <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24">
         <v>0</v>
       </c>
     </row>
@@ -2340,13 +2340,13 @@
         <v>79</v>
       </c>
       <c r="B25">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="C25">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="D25">
-        <v>82.14285714285714</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2354,13 +2354,13 @@
         <v>80</v>
       </c>
       <c r="B26">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C26">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D26">
-        <v>56.52173913043478</v>
+        <v>82.14285714285714</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2368,13 +2368,13 @@
         <v>81</v>
       </c>
       <c r="B27">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C27">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="D27">
-        <v>77.41935483870968</v>
+        <v>56.52173913043478</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2382,13 +2382,13 @@
         <v>82</v>
       </c>
       <c r="B28">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="C28">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="D28">
-        <v>75</v>
+        <v>77.41935483870968</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2396,13 +2396,13 @@
         <v>83</v>
       </c>
       <c r="B29">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C29">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D29">
-        <v>50</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2410,13 +2410,13 @@
         <v>84</v>
       </c>
       <c r="B30">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C30">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D30">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -6089,13 +6089,13 @@
         <v>57</v>
       </c>
       <c r="B3">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C3">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="D3">
-        <v>67.74193548387096</v>
+        <v>92.30769230769231</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -6103,13 +6103,13 @@
         <v>58</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>67.74193548387096</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -6117,13 +6117,13 @@
         <v>59</v>
       </c>
       <c r="B5">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="C5">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -6131,13 +6131,13 @@
         <v>60</v>
       </c>
       <c r="B6">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="C6">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="D6">
-        <v>67.24137931034483</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -6145,13 +6145,13 @@
         <v>61</v>
       </c>
       <c r="B7">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="C7">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="D7">
-        <v>75</v>
+        <v>67.24137931034483</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -6159,13 +6159,13 @@
         <v>62</v>
       </c>
       <c r="B8">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C8">
         <v>16</v>
       </c>
       <c r="D8">
-        <v>68.75</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -6173,13 +6173,13 @@
         <v>63</v>
       </c>
       <c r="B9">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C9">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D9">
-        <v>75</v>
+        <v>68.75</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -6187,13 +6187,13 @@
         <v>64</v>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C10">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D10">
-        <v>45</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -6201,13 +6201,13 @@
         <v>65</v>
       </c>
       <c r="B11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C11">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D11">
-        <v>71.42857142857143</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -6215,13 +6215,13 @@
         <v>66</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D12">
-        <v>100</v>
+        <v>71.42857142857143</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -6229,13 +6229,13 @@
         <v>67</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D13">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -6257,13 +6257,13 @@
         <v>69</v>
       </c>
       <c r="B15">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C15">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="D15">
-        <v>62.26415094339622</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -6271,13 +6271,13 @@
         <v>70</v>
       </c>
       <c r="B16">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="C16">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="D16">
-        <v>72.72727272727273</v>
+        <v>62.26415094339622</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -6285,13 +6285,13 @@
         <v>71</v>
       </c>
       <c r="B17">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C17">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D17">
-        <v>55.55555555555556</v>
+        <v>72.72727272727273</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -6299,13 +6299,13 @@
         <v>72</v>
       </c>
       <c r="B18">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C18">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="D18">
-        <v>76.92307692307693</v>
+        <v>55.55555555555556</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -6313,13 +6313,13 @@
         <v>73</v>
       </c>
       <c r="B19">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C19">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="D19">
-        <v>51.85185185185185</v>
+        <v>76.92307692307693</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -6327,13 +6327,13 @@
         <v>74</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C20">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D20">
-        <v>16.66666666666666</v>
+        <v>51.85185185185185</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -6341,13 +6341,13 @@
         <v>75</v>
       </c>
       <c r="B21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D21">
-        <v>50</v>
+        <v>16.66666666666666</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -6355,13 +6355,13 @@
         <v>76</v>
       </c>
       <c r="B22">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C22">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D22">
-        <v>62.5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -6369,10 +6369,13 @@
         <v>77</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="D23">
+        <v>62.5</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -6383,9 +6386,6 @@
         <v>0</v>
       </c>
       <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24">
         <v>0</v>
       </c>
     </row>
@@ -6394,13 +6394,13 @@
         <v>79</v>
       </c>
       <c r="B25">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="C25">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D25">
-        <v>68.42105263157895</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -6408,13 +6408,13 @@
         <v>80</v>
       </c>
       <c r="B26">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C26">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D26">
-        <v>72.72727272727273</v>
+        <v>68.42105263157895</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -6422,13 +6422,13 @@
         <v>81</v>
       </c>
       <c r="B27">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="C27">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="D27">
-        <v>69.56521739130434</v>
+        <v>72.72727272727273</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -6436,13 +6436,13 @@
         <v>82</v>
       </c>
       <c r="B28">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C28">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="D28">
-        <v>50</v>
+        <v>69.56521739130434</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -6450,13 +6450,13 @@
         <v>83</v>
       </c>
       <c r="B29">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C29">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D29">
-        <v>90.90909090909091</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -6464,13 +6464,13 @@
         <v>84</v>
       </c>
       <c r="B30">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C30">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D30">
-        <v>92.30769230769231</v>
+        <v>90.90909090909091</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -10149,13 +10149,13 @@
         <v>57</v>
       </c>
       <c r="B3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D3">
-        <v>41.37931034482759</v>
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -10163,13 +10163,13 @@
         <v>58</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C4">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="D4">
-        <v>15.38461538461539</v>
+        <v>41.37931034482759</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -10177,13 +10177,13 @@
         <v>59</v>
       </c>
       <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
         <v>13</v>
       </c>
-      <c r="C5">
-        <v>16</v>
-      </c>
       <c r="D5">
-        <v>81.25</v>
+        <v>15.38461538461539</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -10191,13 +10191,13 @@
         <v>60</v>
       </c>
       <c r="B6">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="C6">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="D6">
-        <v>65</v>
+        <v>81.25</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -10205,13 +10205,13 @@
         <v>61</v>
       </c>
       <c r="B7">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="C7">
-        <v>26</v>
+        <v>60</v>
       </c>
       <c r="D7">
-        <v>69.23076923076923</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -10219,13 +10219,13 @@
         <v>62</v>
       </c>
       <c r="B8">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C8">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D8">
-        <v>66.66666666666666</v>
+        <v>69.23076923076923</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -10233,13 +10233,13 @@
         <v>63</v>
       </c>
       <c r="B9">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C9">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D9">
-        <v>60</v>
+        <v>66.66666666666666</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -10247,13 +10247,13 @@
         <v>64</v>
       </c>
       <c r="B10">
+        <v>6</v>
+      </c>
+      <c r="C10">
         <v>10</v>
       </c>
-      <c r="C10">
-        <v>19</v>
-      </c>
       <c r="D10">
-        <v>52.63157894736842</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -10261,13 +10261,13 @@
         <v>65</v>
       </c>
       <c r="B11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="C11">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="D11">
-        <v>89.28571428571429</v>
+        <v>52.63157894736842</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -10275,13 +10275,13 @@
         <v>66</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="D12">
-        <v>50</v>
+        <v>89.28571428571429</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -10289,13 +10289,13 @@
         <v>67</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C13">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D13">
-        <v>36.36363636363637</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -10306,10 +10306,10 @@
         <v>4</v>
       </c>
       <c r="C14">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D14">
-        <v>100</v>
+        <v>36.36363636363637</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -10317,13 +10317,13 @@
         <v>69</v>
       </c>
       <c r="B15">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C15">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="D15">
-        <v>49.12280701754386</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -10331,13 +10331,13 @@
         <v>70</v>
       </c>
       <c r="B16">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="C16">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="D16">
-        <v>69.56521739130434</v>
+        <v>49.12280701754386</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -10345,13 +10345,13 @@
         <v>71</v>
       </c>
       <c r="B17">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C17">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="D17">
-        <v>75</v>
+        <v>69.56521739130434</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -10359,13 +10359,13 @@
         <v>72</v>
       </c>
       <c r="B18">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="C18">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D18">
-        <v>51.72413793103448</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -10373,13 +10373,13 @@
         <v>73</v>
       </c>
       <c r="B19">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C19">
         <v>29</v>
       </c>
       <c r="D19">
-        <v>65.51724137931035</v>
+        <v>51.72413793103448</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -10387,13 +10387,13 @@
         <v>74</v>
       </c>
       <c r="B20">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="C20">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="D20">
-        <v>77.77777777777779</v>
+        <v>65.51724137931035</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -10401,13 +10401,13 @@
         <v>75</v>
       </c>
       <c r="B21">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C21">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D21">
-        <v>80</v>
+        <v>77.77777777777779</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -10415,13 +10415,13 @@
         <v>76</v>
       </c>
       <c r="B22">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C22">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="D22">
-        <v>68.18181818181817</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -10429,13 +10429,13 @@
         <v>77</v>
       </c>
       <c r="B23">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C23">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D23">
-        <v>46.66666666666666</v>
+        <v>68.18181818181817</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -10443,10 +10443,13 @@
         <v>78</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="D24">
+        <v>46.66666666666666</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -10454,13 +10457,10 @@
         <v>79</v>
       </c>
       <c r="B25">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="C25">
-        <v>21</v>
-      </c>
-      <c r="D25">
-        <v>61.90476190476191</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -10468,13 +10468,13 @@
         <v>80</v>
       </c>
       <c r="B26">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C26">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D26">
-        <v>64</v>
+        <v>61.90476190476191</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -10482,13 +10482,13 @@
         <v>81</v>
       </c>
       <c r="B27">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="C27">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="D27">
-        <v>43.54838709677419</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -10496,13 +10496,13 @@
         <v>82</v>
       </c>
       <c r="B28">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="C28">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="D28">
-        <v>60</v>
+        <v>43.54838709677419</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -10510,13 +10510,13 @@
         <v>83</v>
       </c>
       <c r="B29">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C29">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D29">
-        <v>77.77777777777779</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -10524,13 +10524,13 @@
         <v>84</v>
       </c>
       <c r="B30">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C30">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="D30">
-        <v>43.33333333333334</v>
+        <v>77.77777777777779</v>
       </c>
     </row>
     <row r="31" spans="1:4">

</xml_diff>